<commit_message>
feat(invoices): email payment reminder from the All invoices page [INV-004]
A Send email reminder button on every Outstanding invoice opens a drafted, editable email to the stored Customer Email; sending records the reminder and shows Last reminder sent. Adds the optional Customer Email column to uploads and the template, a Mailpit service as the default mail sink, SMTP settings, a reusable Dialog and InlineAlert, and moves the Record status under the invoice number so the table fits 1280px. Reminder emails are plain text, never logged, and only ever sent to the stored address.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/invoices-sample.xlsx
+++ b/samples/invoices-sample.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -441,6 +441,7 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,6 +475,11 @@
           <t>Paid Date</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Customer Email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -487,16 +493,21 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46215</v>
+        <v>46225</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>46245</v>
+        <v>46255</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>185000</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>46240</v>
+        <v>46250</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>accounts@sharmatextiles.example</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -511,16 +522,21 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>46230</v>
+        <v>46240</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>46260</v>
+        <v>46270</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>42750.5</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>46262</v>
+        <v>46272</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>payables@kaveriagro.example</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -535,16 +551,21 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>46250</v>
+        <v>46260</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>46280</v>
+        <v>46290</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>96400</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>46278</v>
+        <v>46288</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ap@bluewavelogistics.example</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -559,16 +580,21 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>46270</v>
+        <v>46280</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>46300</v>
+        <v>46310</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>310000</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>46288</v>
+        <v>46298</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>accounts@mehtaauto.example</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -583,16 +609,21 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>46275</v>
+        <v>46285</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>46292</v>
+        <v>46302</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>18500</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>46289</v>
+        <v>46299</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>finance@greenleaf.example</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -607,15 +638,20 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>46220</v>
+        <v>46230</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>46250</v>
+        <v>46260</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>125000</v>
       </c>
       <c r="F7" s="2" t="n"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>accounts@deccanprinting.example</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -629,15 +665,20 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>46245</v>
+        <v>46255</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>46275</v>
+        <v>46285</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>267500.75</v>
       </c>
       <c r="F8" s="2" t="n"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ap@sunrisepharma.example</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -651,10 +692,10 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>46255</v>
+        <v>46265</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>46285</v>
+        <v>46295</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>54000</v>
@@ -673,15 +714,20 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>46259</v>
+        <v>46269</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>46289</v>
+        <v>46299</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>8900</v>
       </c>
       <c r="F10" s="2" t="n"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>payables@kaveriagro.example</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -695,15 +741,20 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>46260</v>
+        <v>46270</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>46290</v>
+        <v>46300</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>142000</v>
       </c>
       <c r="F11" s="2" t="n"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>accounts@mehtaauto.example</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -717,15 +768,20 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>46262</v>
+        <v>46272</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>46291</v>
+        <v>46301</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>76250</v>
       </c>
       <c r="F12" s="2" t="n"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ap@bluewavelogistics.example</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -739,15 +795,20 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>46263</v>
+        <v>46273</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>46293</v>
+        <v>46303</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>225000</v>
       </c>
       <c r="F13" s="2" t="n"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>accounts@sharmatextiles.example</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -761,15 +822,20 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>46265</v>
+        <v>46275</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>46295</v>
+        <v>46305</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>31500</v>
       </c>
       <c r="F14" s="2" t="n"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>finance@greenleaf.example</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -783,15 +849,20 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>46270</v>
+        <v>46280</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>46296</v>
+        <v>46306</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>64000</v>
       </c>
       <c r="F15" s="2" t="n"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>accounts@deccanprinting.example</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -805,15 +876,20 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>46280</v>
+        <v>46290</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>46310</v>
+        <v>46320</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>410000</v>
       </c>
       <c r="F16" s="2" t="n"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>ap@sunrisepharma.example</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -827,10 +903,10 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>46285</v>
+        <v>46295</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>46315</v>
+        <v>46325</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>22800</v>
@@ -849,15 +925,20 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>46288</v>
+        <v>46298</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>46335</v>
+        <v>46345</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>98000</v>
       </c>
       <c r="F18" s="2" t="n"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>payables@kaveriagro.example</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1096,7 +1177,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Generated on 25 September 2026. Only the first sheet is read on upload.</t>
+          <t>Generated on 5 October 2026. Only the first sheet is read on upload.</t>
         </is>
       </c>
     </row>

</xml_diff>